<commit_message>
Updated scripts in \apps, \core, default_dataset_409.xlsx, .gitignore.
</commit_message>
<xml_diff>
--- a/data/defaults/default_dataset_409.xlsx
+++ b/data/defaults/default_dataset_409.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sammo\My_Documents\Programming\Python_Programs\Sun_Chemical\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sammo\Projects\SunChemicalUrethaneRecommender\data\defaults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4048198E-B9E7-4889-B22D-B242DB7831AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D35223E-D67E-4819-B09E-CE6176522486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>